<commit_message>
Fix: remove locked_out_user from test data
</commit_message>
<xml_diff>
--- a/testdata/LoginData.xlsx
+++ b/testdata/LoginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ashish\IdeaProjects\EcommerceAutomationFramework\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3E2E9173-3F51-4F62-8A70-02953A50D2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B000A283-3BD9-4D51-A04D-D88AF3E4849A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{111A513E-B010-4CB5-B5ED-3BCE076866F4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>username</t>
   </si>
@@ -48,9 +48,6 @@
   </si>
   <si>
     <t>secret_sauce</t>
-  </si>
-  <si>
-    <t>locked_out_user</t>
   </si>
   <si>
     <t>problem_user</t>
@@ -439,7 +436,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0CD7CD8-14D1-4EAA-A291-84A28EBD376E}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="14.9296875" customWidth="1"/>
@@ -462,19 +459,11 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="28.5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A4" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>